<commit_message>
Populate Sheet 4 (Cashflow Statement) and Sheet 5 (DCF Valuation & Sensitivity Matrix) in Excel file
</commit_message>
<xml_diff>
--- a/NexGen_Tech_Financial_Model_and_DCF_Valuation.xlsx
+++ b/NexGen_Tech_Financial_Model_and_DCF_Valuation.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/062d628e8a33ccc6/Documents/Projects/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\omkar\OneDrive\Documents\Portfolio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{017AE41E-2AA9-4170-8A34-6A6B6BD90768}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CABC62D-E700-4161-BBFE-2C3DCA7D464E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A35E1EFC-E7D2-4244-B9C6-69BD6C11D796}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="94">
   <si>
     <t>NEXGEN TECH PVT LTD — MODEL ASSUMPTIONS &amp; DRIVERS</t>
   </si>
@@ -244,17 +244,99 @@
   </si>
   <si>
     <t>TOTAL NON-CURRENT LIABILITIES</t>
+  </si>
+  <si>
+    <t>NEXGEN TECH - PRO FORMA STATEMENT OF CASH FLOWS (2026 - 2029)</t>
+  </si>
+  <si>
+    <t>Cash Flow Statement Line Item</t>
+  </si>
+  <si>
+    <t>CASH FLOW FROM OPERATING ACTIVITIES</t>
+  </si>
+  <si>
+    <t>Net Income (PAT)</t>
+  </si>
+  <si>
+    <t>Add: Non-Cash Depreciation</t>
+  </si>
+  <si>
+    <t>Change in Working Capital (AR &amp; AP)</t>
+  </si>
+  <si>
+    <t>CASH FLOW FROM OPERATIONS (CFO)</t>
+  </si>
+  <si>
+    <t>CASH FLOW FROM INVESTING ACTIVITIES</t>
+  </si>
+  <si>
+    <t>Capital Expenditures (CapEx)</t>
+  </si>
+  <si>
+    <t>CASH FLOW FROM INVESTING (CFI)</t>
+  </si>
+  <si>
+    <t>CASH FLOW FROM FINANCING ACTIVITIES</t>
+  </si>
+  <si>
+    <t>Long-Term Debt Repayment / Issuance</t>
+  </si>
+  <si>
+    <t>CASH FLOW FROM FINANCING (CFF)</t>
+  </si>
+  <si>
+    <t>NET CHANGE IN CASH BALANCE</t>
+  </si>
+  <si>
+    <t>Beginning Cash Balance</t>
+  </si>
+  <si>
+    <t>ENDING CASH BALANCE</t>
+  </si>
+  <si>
+    <t>NEXGEN TECH - DCF VALUATION &amp; TWO-WAY SENSITIVITY MATRIX</t>
+  </si>
+  <si>
+    <t>VALUATION PARAMETER</t>
+  </si>
+  <si>
+    <t>VALUE</t>
+  </si>
+  <si>
+    <t>Base 2029 Forecast EBITDA</t>
+  </si>
+  <si>
+    <t>Effective Tax Rate</t>
+  </si>
+  <si>
+    <t>Weighted Average Cost of Capital (WACC)</t>
+  </si>
+  <si>
+    <t>Terminal Growth Rate (g)</t>
+  </si>
+  <si>
+    <t>IMPLIED ENTERPRISE VALUE</t>
+  </si>
+  <si>
+    <t>TWO-WAY DCF VALUATION SENSITIVITY MATRIX</t>
+  </si>
+  <si>
+    <t>IMPLIED ENTERPRISE VALUE: â‚¹ 1,92,38,543</t>
+  </si>
+  <si>
+    <t>WACC \ Terminal Growth (g)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="5" formatCode="&quot;₹&quot;\ #,##0;&quot;₹&quot;\ \-#,##0"/>
     <numFmt numFmtId="44" formatCode="_ &quot;₹&quot;\ * #,##0.00_ ;_ &quot;₹&quot;\ * \-#,##0.00_ ;_ &quot;₹&quot;\ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -372,8 +454,24 @@
       <family val="2"/>
       <scheme val="major"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -410,6 +508,42 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF141926"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE6F9DD"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC7F3FE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFEEADB"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDF9E6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF9E6DD"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -440,45 +574,21 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="5" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="5" fontId="9" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="5" fontId="11" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="9" fontId="10" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="5" fontId="9" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="5" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="5" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="5" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -488,7 +598,7 @@
     <xf numFmtId="9" fontId="11" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="11" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="11" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="5" fontId="11" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -526,9 +636,50 @@
     <xf numFmtId="9" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="16" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="2" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="3" fontId="2" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="3" fontId="2" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="3" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="3" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="3" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="9" fontId="15" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -874,239 +1025,239 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="48" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4"/>
+      <c r="B1" s="48"/>
     </row>
     <row r="2" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="4"/>
-      <c r="B2" s="4"/>
+      <c r="A2" s="48"/>
+      <c r="B2" s="48"/>
     </row>
     <row r="3" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
     </row>
     <row r="4" spans="1:5" ht="19.2" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="47" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="3"/>
+      <c r="B4" s="47"/>
       <c r="C4" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="22" t="s">
+      <c r="A6" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="22" t="s">
+      <c r="B6" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="34" t="s">
+      <c r="C6" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="35" t="s">
+      <c r="D6" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="E6" s="22" t="s">
+      <c r="E6" s="14" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="23" t="s">
+      <c r="A7" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="24">
+      <c r="B7" s="16">
         <v>0.25</v>
       </c>
-      <c r="C7" s="24">
+      <c r="C7" s="16">
         <v>0.35</v>
       </c>
-      <c r="D7" s="24">
+      <c r="D7" s="16">
         <v>0.1</v>
       </c>
-      <c r="E7" s="25">
+      <c r="E7" s="17">
         <f>CHOOSE($C$4, B7, C7, D7)</f>
         <v>0.25</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="23" t="s">
+      <c r="A8" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="24">
+      <c r="B8" s="16">
         <v>0.2</v>
       </c>
-      <c r="C8" s="24">
+      <c r="C8" s="16">
         <v>0.16</v>
       </c>
-      <c r="D8" s="24">
+      <c r="D8" s="16">
         <v>0.25</v>
       </c>
-      <c r="E8" s="25">
-        <f t="shared" ref="E8:E14" si="0">CHOOSE($C$4, B8, C8, D8)</f>
+      <c r="E8" s="17">
+        <f t="shared" ref="E8:E13" si="0">CHOOSE($C$4, B8, C8, D8)</f>
         <v>0.2</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="23" t="s">
+      <c r="A9" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="24">
+      <c r="B9" s="16">
         <v>0.25</v>
       </c>
-      <c r="C9" s="24">
+      <c r="C9" s="16">
         <v>0.2</v>
       </c>
-      <c r="D9" s="24">
+      <c r="D9" s="16">
         <v>0.3</v>
       </c>
-      <c r="E9" s="25">
+      <c r="E9" s="17">
         <f t="shared" si="0"/>
         <v>0.25</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A10" s="23" t="s">
+      <c r="A10" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="24">
+      <c r="B10" s="16">
         <v>0.18</v>
       </c>
-      <c r="C10" s="24">
+      <c r="C10" s="16">
         <v>0.15</v>
       </c>
-      <c r="D10" s="24">
+      <c r="D10" s="16">
         <v>0.22</v>
       </c>
-      <c r="E10" s="25">
+      <c r="E10" s="17">
         <f t="shared" si="0"/>
         <v>0.18</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="23" t="s">
+      <c r="A11" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="24">
+      <c r="B11" s="16">
         <v>0.08</v>
       </c>
-      <c r="C11" s="24">
+      <c r="C11" s="16">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="D11" s="24">
+      <c r="D11" s="16">
         <v>0.1</v>
       </c>
-      <c r="E11" s="25">
+      <c r="E11" s="17">
         <f t="shared" si="0"/>
         <v>0.08</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="23" t="s">
+      <c r="A12" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="26">
+      <c r="B12" s="18">
         <v>600000</v>
       </c>
-      <c r="C12" s="26">
+      <c r="C12" s="18">
         <v>600000</v>
       </c>
-      <c r="D12" s="26">
+      <c r="D12" s="18">
         <v>650000</v>
       </c>
-      <c r="E12" s="27">
+      <c r="E12" s="19">
         <f t="shared" si="0"/>
         <v>600000</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A13" s="23" t="s">
+      <c r="A13" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="24">
+      <c r="B13" s="16">
         <v>0.25</v>
       </c>
-      <c r="C13" s="24">
+      <c r="C13" s="16">
         <v>0.25</v>
       </c>
-      <c r="D13" s="24">
+      <c r="D13" s="16">
         <v>0.25</v>
       </c>
-      <c r="E13" s="25">
+      <c r="E13" s="17">
         <f t="shared" si="0"/>
         <v>0.25</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="23" t="s">
+      <c r="A14" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="B14" s="24">
+      <c r="B14" s="16">
         <v>0.1</v>
       </c>
-      <c r="C14" s="24">
+      <c r="C14" s="16">
         <v>0.1</v>
       </c>
-      <c r="D14" s="24">
+      <c r="D14" s="16">
         <v>0.1</v>
       </c>
-      <c r="E14" s="25">
+      <c r="E14" s="17">
         <f>CHOOSE($C$4, B14, C14, D14)</f>
         <v>0.1</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="28" t="s">
+      <c r="A15" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="B15" s="29">
+      <c r="B15" s="21">
         <v>1000000</v>
       </c>
-      <c r="C15" s="36">
+      <c r="C15" s="28">
         <v>1000000</v>
       </c>
-      <c r="D15" s="36">
+      <c r="D15" s="28">
         <v>1000000</v>
       </c>
-      <c r="E15" s="29">
+      <c r="E15" s="21">
         <f>CHOOSE($C$4, B15,C15,D15)</f>
         <v>1000000</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A16" s="30" t="s">
+      <c r="A16" s="22" t="s">
         <v>38</v>
       </c>
-      <c r="B16" s="31">
+      <c r="B16" s="23">
         <v>625000</v>
       </c>
-      <c r="C16" s="37">
+      <c r="C16" s="29">
         <v>625000</v>
       </c>
-      <c r="D16" s="37">
+      <c r="D16" s="29">
         <v>625000</v>
       </c>
-      <c r="E16" s="31">
+      <c r="E16" s="23">
         <f>CHOOSE($C$4, B16, C16, D16)</f>
         <v>625000</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A17" s="30" t="s">
+      <c r="A17" s="22" t="s">
         <v>39</v>
       </c>
-      <c r="B17" s="32">
+      <c r="B17" s="24">
         <v>0.08</v>
       </c>
-      <c r="C17" s="38">
+      <c r="C17" s="30">
         <v>0.08</v>
       </c>
-      <c r="D17" s="38">
+      <c r="D17" s="30">
         <v>0.08</v>
       </c>
-      <c r="E17" s="33">
+      <c r="E17" s="25">
         <f>CHOOSE($C$4, B17, C17, D17)</f>
         <v>0.08</v>
       </c>
@@ -1135,367 +1286,367 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="50" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
+      <c r="B1" s="50"/>
+      <c r="C1" s="50"/>
+      <c r="D1" s="50"/>
     </row>
     <row r="2" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="10"/>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
+      <c r="A2" s="50"/>
+      <c r="B2" s="50"/>
+      <c r="C2" s="50"/>
+      <c r="D2" s="50"/>
     </row>
     <row r="5" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="51" t="s">
         <v>36</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="52" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="21" t="s">
+      <c r="C5" s="49" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="21" t="s">
+      <c r="D5" s="49" t="s">
         <v>18</v>
       </c>
-      <c r="E5" s="21" t="s">
+      <c r="E5" s="49" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" s="19"/>
-      <c r="B6" s="20"/>
-      <c r="C6" s="21"/>
-      <c r="D6" s="21"/>
-      <c r="E6" s="21"/>
+      <c r="A6" s="51"/>
+      <c r="B6" s="52"/>
+      <c r="C6" s="49"/>
+      <c r="D6" s="49"/>
+      <c r="E6" s="49"/>
     </row>
     <row r="7" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B7" s="7">
+      <c r="B7" s="5">
         <v>5000000</v>
       </c>
-      <c r="C7" s="9">
+      <c r="C7" s="7">
         <f>B7 * (1 + Assumptions!$E$7)</f>
         <v>6250000</v>
       </c>
-      <c r="D7" s="9">
+      <c r="D7" s="7">
         <f>C7 * (1 + Assumptions!$E$7)</f>
         <v>7812500</v>
       </c>
-      <c r="E7" s="9">
+      <c r="E7" s="7">
         <f>D7 * (1 + Assumptions!$E$7)</f>
         <v>9765625</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="7">
+      <c r="B8" s="5">
         <v>1000000</v>
       </c>
-      <c r="C8" s="7">
+      <c r="C8" s="5">
         <f>C7*Assumptions!$E$8</f>
         <v>1250000</v>
       </c>
-      <c r="D8" s="7">
+      <c r="D8" s="5">
         <f>D7*Assumptions!$E$8</f>
         <v>1562500</v>
       </c>
-      <c r="E8" s="7">
+      <c r="E8" s="5">
         <f>E7*Assumptions!$E$8</f>
         <v>1953125</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="8">
+      <c r="B9" s="6">
         <f>B7-B8</f>
         <v>4000000</v>
       </c>
-      <c r="C9" s="8">
+      <c r="C9" s="6">
         <f>C7-C8</f>
         <v>5000000</v>
       </c>
-      <c r="D9" s="8">
+      <c r="D9" s="6">
         <f t="shared" ref="D9:E9" si="0">D7-D8</f>
         <v>6250000</v>
       </c>
-      <c r="E9" s="8">
+      <c r="E9" s="6">
         <f t="shared" si="0"/>
         <v>7812500</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
     </row>
     <row r="11" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B11" s="7">
+      <c r="B11" s="5">
         <v>1250000</v>
       </c>
-      <c r="C11" s="7">
+      <c r="C11" s="5">
         <f>C7*Assumptions!$E$9</f>
         <v>1562500</v>
       </c>
-      <c r="D11" s="7">
+      <c r="D11" s="5">
         <f>D7*Assumptions!$E$9</f>
         <v>1953125</v>
       </c>
-      <c r="E11" s="7">
+      <c r="E11" s="5">
         <f>E7*Assumptions!$E$9</f>
         <v>2441406.25</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B12" s="7">
+      <c r="B12" s="5">
         <v>900000</v>
       </c>
-      <c r="C12" s="7">
+      <c r="C12" s="5">
         <f>C7*Assumptions!$E$10</f>
         <v>1125000</v>
       </c>
-      <c r="D12" s="7">
+      <c r="D12" s="5">
         <f>D7*Assumptions!$E$10</f>
         <v>1406250</v>
       </c>
-      <c r="E12" s="7">
+      <c r="E12" s="5">
         <f>E7*Assumptions!$E$10</f>
         <v>1757812.5</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A13" s="5" t="s">
+      <c r="A13" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B13" s="7">
+      <c r="B13" s="5">
         <v>400000</v>
       </c>
-      <c r="C13" s="7">
+      <c r="C13" s="5">
         <f>C7*Assumptions!$E$11</f>
         <v>500000</v>
       </c>
-      <c r="D13" s="7">
+      <c r="D13" s="5">
         <f>D7*Assumptions!$E$11</f>
         <v>625000</v>
       </c>
-      <c r="E13" s="7">
+      <c r="E13" s="5">
         <f>E7*Assumptions!$E$11</f>
         <v>781250</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="7">
+      <c r="B14" s="5">
         <v>600000</v>
       </c>
-      <c r="C14" s="7">
+      <c r="C14" s="5">
         <f>Assumptions!$E$12</f>
         <v>600000</v>
       </c>
-      <c r="D14" s="7">
+      <c r="D14" s="5">
         <f>Assumptions!$E$12</f>
         <v>600000</v>
       </c>
-      <c r="E14" s="7">
+      <c r="E14" s="5">
         <f>Assumptions!$E$12</f>
         <v>600000</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="6" t="s">
+      <c r="A15" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B15" s="8">
+      <c r="B15" s="6">
         <f>SUM(B11:B14)</f>
         <v>3150000</v>
       </c>
-      <c r="C15" s="8">
+      <c r="C15" s="6">
         <f>SUM(C11:C14)</f>
         <v>3787500</v>
       </c>
-      <c r="D15" s="8">
+      <c r="D15" s="6">
         <f t="shared" ref="D15:E15" si="1">SUM(D11:D14)</f>
         <v>4584375</v>
       </c>
-      <c r="E15" s="8">
+      <c r="E15" s="6">
         <f t="shared" si="1"/>
         <v>5580468.75</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A16" s="6" t="s">
+      <c r="A16" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B16" s="8">
+      <c r="B16" s="6">
         <f>B9-B15</f>
         <v>850000</v>
       </c>
-      <c r="C16" s="8">
+      <c r="C16" s="6">
         <f>C9-C15</f>
         <v>1212500</v>
       </c>
-      <c r="D16" s="8">
+      <c r="D16" s="6">
         <f t="shared" ref="D16:E16" si="2">D9-D15</f>
         <v>1665625</v>
       </c>
-      <c r="E16" s="8">
+      <c r="E16" s="6">
         <f t="shared" si="2"/>
         <v>2232031.25</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A17" s="5" t="s">
+      <c r="A17" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B17" s="7">
+      <c r="B17" s="5">
         <v>100000</v>
       </c>
-      <c r="C17" s="7">
+      <c r="C17" s="5">
         <f>Assumptions!$E$15*Assumptions!$E$14</f>
         <v>100000</v>
       </c>
-      <c r="D17" s="7">
+      <c r="D17" s="5">
         <f>Assumptions!$E$15*Assumptions!$E$14</f>
         <v>100000</v>
       </c>
-      <c r="E17" s="7">
+      <c r="E17" s="5">
         <f>Assumptions!$E$15*Assumptions!$E$14</f>
         <v>100000</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A18" s="6" t="s">
+      <c r="A18" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B18" s="8">
+      <c r="B18" s="6">
         <f>B16-B17</f>
         <v>750000</v>
       </c>
-      <c r="C18" s="8">
+      <c r="C18" s="6">
         <f>C16-C17</f>
         <v>1112500</v>
       </c>
-      <c r="D18" s="8">
+      <c r="D18" s="6">
         <f t="shared" ref="D18:E18" si="3">D16-D17</f>
         <v>1565625</v>
       </c>
-      <c r="E18" s="8">
+      <c r="E18" s="6">
         <f t="shared" si="3"/>
         <v>2132031.25</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A19" s="5" t="s">
+      <c r="A19" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B19" s="7">
+      <c r="B19" s="5">
         <v>50000</v>
       </c>
-      <c r="C19" s="7">
+      <c r="C19" s="5">
         <f>Assumptions!$E$16*Assumptions!$E$17</f>
         <v>50000</v>
       </c>
-      <c r="D19" s="7">
+      <c r="D19" s="5">
         <f>Assumptions!$E$16*Assumptions!$E$17</f>
         <v>50000</v>
       </c>
-      <c r="E19" s="7">
+      <c r="E19" s="5">
         <f>Assumptions!$E$16*Assumptions!$E$17</f>
         <v>50000</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A20" s="6" t="s">
+      <c r="A20" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B20" s="8">
+      <c r="B20" s="6">
         <f>B18-B19</f>
         <v>700000</v>
       </c>
-      <c r="C20" s="8">
+      <c r="C20" s="6">
         <f>C18-C19</f>
         <v>1062500</v>
       </c>
-      <c r="D20" s="8">
+      <c r="D20" s="6">
         <f t="shared" ref="D20:E20" si="4">D18-D19</f>
         <v>1515625</v>
       </c>
-      <c r="E20" s="8">
+      <c r="E20" s="6">
         <f t="shared" si="4"/>
         <v>2082031.25</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A21" s="5" t="s">
+      <c r="A21" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B21" s="7">
+      <c r="B21" s="5">
         <f>B20*0.25</f>
         <v>175000</v>
       </c>
-      <c r="C21" s="7">
+      <c r="C21" s="5">
         <f>IF(C20&gt;0,C20*Assumptions!$E$13,0)</f>
         <v>265625</v>
       </c>
-      <c r="D21" s="7">
+      <c r="D21" s="5">
         <f>IF(D20&gt;0,D20*Assumptions!$E$13,0)</f>
         <v>378906.25</v>
       </c>
-      <c r="E21" s="7">
+      <c r="E21" s="5">
         <f>IF(E20&gt;0,E20*Assumptions!$E$13,0)</f>
         <v>520507.8125</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A22" s="14" t="s">
+      <c r="A22" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B22" s="15">
+      <c r="B22" s="10">
         <f>B20-B21</f>
         <v>525000</v>
       </c>
-      <c r="C22" s="15">
+      <c r="C22" s="10">
         <f>C20-C21</f>
         <v>796875</v>
       </c>
-      <c r="D22" s="15">
+      <c r="D22" s="10">
         <f t="shared" ref="D22:E22" si="5">D20-D21</f>
         <v>1136718.75</v>
       </c>
-      <c r="E22" s="15">
+      <c r="E22" s="10">
         <f t="shared" si="5"/>
         <v>1561523.4375</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="E5:E6"/>
     <mergeCell ref="A1:D2"/>
     <mergeCell ref="A5:A6"/>
     <mergeCell ref="B5:B6"/>
     <mergeCell ref="C5:C6"/>
     <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -1516,475 +1667,475 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="53" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
+      <c r="B1" s="53"/>
+      <c r="C1" s="53"/>
+      <c r="D1" s="53"/>
+      <c r="E1" s="53"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
     </row>
     <row r="2" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="39"/>
-      <c r="B2" s="39"/>
-      <c r="C2" s="39"/>
-      <c r="D2" s="39"/>
-      <c r="E2" s="39"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13"/>
+      <c r="A2" s="53"/>
+      <c r="B2" s="53"/>
+      <c r="C2" s="53"/>
+      <c r="D2" s="53"/>
+      <c r="E2" s="53"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
     </row>
     <row r="3" spans="1:7" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="54" t="s">
         <v>41</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="54" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="C3" s="55" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="12" t="s">
+      <c r="D3" s="55" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="12" t="s">
+      <c r="E3" s="55" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="11"/>
-      <c r="B4" s="11"/>
-      <c r="C4" s="12"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="12"/>
+      <c r="A4" s="54"/>
+      <c r="B4" s="54"/>
+      <c r="C4" s="55"/>
+      <c r="D4" s="55"/>
+      <c r="E4" s="55"/>
     </row>
     <row r="5" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="4" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="B6" s="5"/>
+      <c r="B6" s="3"/>
     </row>
     <row r="7" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B7" s="7">
+      <c r="B7" s="5">
         <v>1500000</v>
       </c>
-      <c r="C7" s="16">
+      <c r="C7" s="11">
         <f>C32-C15-C8</f>
         <v>2520162.0958904112</v>
       </c>
-      <c r="D7" s="16">
+      <c r="D7" s="11">
         <f>D32-D15-D8</f>
         <v>3654141.1198630137</v>
       </c>
-      <c r="E7" s="16">
-        <f t="shared" ref="D7:E7" si="0">E32-E15-E8</f>
+      <c r="E7" s="11">
+        <f t="shared" ref="E7" si="0">E32-E15-E8</f>
         <v>5187239.8998287665</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B8" s="7">
+      <c r="B8" s="5">
         <v>616438</v>
       </c>
-      <c r="C8" s="16">
+      <c r="C8" s="11">
         <f>('Income statement '!C7/365)*30</f>
         <v>513698.63013698626</v>
       </c>
-      <c r="D8" s="16">
+      <c r="D8" s="11">
         <f>('Income statement '!D7/365)*30</f>
         <v>642123.28767123283</v>
       </c>
-      <c r="E8" s="16">
+      <c r="E8" s="11">
         <f>('Income statement '!E7/365)*30</f>
         <v>802654.10958904109</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="B9" s="8">
+      <c r="B9" s="6">
         <f>SUM(B7:B8)</f>
         <v>2116438</v>
       </c>
-      <c r="C9" s="18">
+      <c r="C9" s="13">
         <f>SUM(C7:C8)</f>
         <v>3033860.7260273974</v>
       </c>
-      <c r="D9" s="18">
+      <c r="D9" s="13">
         <f t="shared" ref="D9:E9" si="1">SUM(D7:D8)</f>
         <v>4296264.4075342463</v>
       </c>
-      <c r="E9" s="18">
+      <c r="E9" s="13">
         <f t="shared" si="1"/>
         <v>5989894.0094178077</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A10" s="5"/>
-      <c r="B10" s="7"/>
+      <c r="A10" s="3"/>
+      <c r="B10" s="5"/>
     </row>
     <row r="11" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="6" t="s">
+      <c r="A11" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="B11" s="7"/>
+      <c r="B11" s="5"/>
     </row>
     <row r="12" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="B12" s="7">
+      <c r="B12" s="5">
         <v>1000000</v>
       </c>
-      <c r="C12" s="16">
+      <c r="C12" s="11">
         <f>B12</f>
         <v>1000000</v>
       </c>
-      <c r="D12" s="16">
+      <c r="D12" s="11">
         <f t="shared" ref="D12:E12" si="2">C12</f>
         <v>1000000</v>
       </c>
-      <c r="E12" s="16">
+      <c r="E12" s="11">
         <f t="shared" si="2"/>
         <v>1000000</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A13" s="5" t="s">
+      <c r="A13" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="B13" s="7">
+      <c r="B13" s="5">
         <v>100000</v>
       </c>
-      <c r="C13" s="16">
+      <c r="C13" s="11">
         <f>B13+'Income statement '!C17</f>
         <v>200000</v>
       </c>
-      <c r="D13" s="16">
+      <c r="D13" s="11">
         <f>C13+'Income statement '!D17</f>
         <v>300000</v>
       </c>
-      <c r="E13" s="16">
+      <c r="E13" s="11">
         <f>D13+'Income statement '!E17</f>
         <v>400000</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="B14" s="7">
+      <c r="B14" s="5">
         <f>B12-B13</f>
         <v>900000</v>
       </c>
-      <c r="C14" s="16">
+      <c r="C14" s="11">
         <f>C12-C13</f>
         <v>800000</v>
       </c>
-      <c r="D14" s="16">
+      <c r="D14" s="11">
         <f t="shared" ref="D14:E14" si="3">D12-D13</f>
         <v>700000</v>
       </c>
-      <c r="E14" s="16">
+      <c r="E14" s="11">
         <f t="shared" si="3"/>
         <v>600000</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="6" t="s">
+      <c r="A15" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="B15" s="8">
+      <c r="B15" s="6">
         <f>B14</f>
         <v>900000</v>
       </c>
-      <c r="C15" s="16">
+      <c r="C15" s="11">
         <f>C14</f>
         <v>800000</v>
       </c>
-      <c r="D15" s="16">
+      <c r="D15" s="11">
         <f t="shared" ref="D15:E15" si="4">D14</f>
         <v>700000</v>
       </c>
-      <c r="E15" s="16">
+      <c r="E15" s="11">
         <f t="shared" si="4"/>
         <v>600000</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A16" s="14" t="s">
+      <c r="A16" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="B16" s="15">
+      <c r="B16" s="10">
         <f>B9+B14</f>
         <v>3016438</v>
       </c>
-      <c r="C16" s="17">
+      <c r="C16" s="12">
         <f>C9+C15</f>
         <v>3833860.7260273974</v>
       </c>
-      <c r="D16" s="17">
+      <c r="D16" s="12">
         <f t="shared" ref="D16:E16" si="5">D9+D15</f>
         <v>4996264.4075342463</v>
       </c>
-      <c r="E16" s="17">
+      <c r="E16" s="12">
         <f t="shared" si="5"/>
         <v>6589894.0094178077</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A17" s="5"/>
-      <c r="B17" s="7"/>
+      <c r="A17" s="3"/>
+      <c r="B17" s="5"/>
     </row>
     <row r="18" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A18" s="6" t="s">
+      <c r="A18" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="B18" s="7"/>
+      <c r="B18" s="5"/>
     </row>
     <row r="19" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A19" s="6" t="s">
+      <c r="A19" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="B19" s="7"/>
+      <c r="B19" s="5"/>
     </row>
     <row r="20" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A20" s="5" t="s">
+      <c r="A20" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="B20" s="7">
+      <c r="B20" s="5">
         <v>82192</v>
       </c>
-      <c r="C20" s="16">
+      <c r="C20" s="11">
         <f>('Income statement '!C8/365)*30</f>
         <v>102739.72602739726</v>
       </c>
-      <c r="D20" s="16">
+      <c r="D20" s="11">
         <f>('Income statement '!D8/365)*30</f>
         <v>128424.65753424657</v>
       </c>
-      <c r="E20" s="16">
+      <c r="E20" s="11">
         <f>('Income statement '!E8/365)*30</f>
         <v>160530.82191780821</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A21" s="6" t="s">
+      <c r="A21" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="B21" s="8">
+      <c r="B21" s="6">
         <f>B20</f>
         <v>82192</v>
       </c>
-      <c r="C21" s="18">
+      <c r="C21" s="13">
         <f>C20</f>
         <v>102739.72602739726</v>
       </c>
-      <c r="D21" s="18">
+      <c r="D21" s="13">
         <f t="shared" ref="D21:E21" si="6">D20</f>
         <v>128424.65753424657</v>
       </c>
-      <c r="E21" s="18">
+      <c r="E21" s="13">
         <f t="shared" si="6"/>
         <v>160530.82191780821</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A22" s="5"/>
-      <c r="B22" s="7"/>
+      <c r="A22" s="3"/>
+      <c r="B22" s="5"/>
     </row>
     <row r="23" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A23" s="5" t="s">
+      <c r="A23" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="B23" s="7"/>
+      <c r="B23" s="5"/>
     </row>
     <row r="24" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A24" s="5" t="s">
+      <c r="A24" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="B24" s="7">
+      <c r="B24" s="5">
         <v>625000</v>
       </c>
-      <c r="C24" s="16">
+      <c r="C24" s="11">
         <f>B24</f>
         <v>625000</v>
       </c>
-      <c r="D24" s="16">
+      <c r="D24" s="11">
         <f t="shared" ref="D24:E24" si="7">C24</f>
         <v>625000</v>
       </c>
-      <c r="E24" s="16">
+      <c r="E24" s="11">
         <f t="shared" si="7"/>
         <v>625000</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A25" s="6" t="s">
+      <c r="A25" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="B25" s="7">
+      <c r="B25" s="5">
         <f>B24</f>
         <v>625000</v>
       </c>
-      <c r="C25" s="16">
+      <c r="C25" s="11">
         <f>C24</f>
         <v>625000</v>
       </c>
-      <c r="D25" s="16">
+      <c r="D25" s="11">
         <f t="shared" ref="D25:E25" si="8">D24</f>
         <v>625000</v>
       </c>
-      <c r="E25" s="16">
+      <c r="E25" s="11">
         <f t="shared" si="8"/>
         <v>625000</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A26" s="6" t="s">
+      <c r="A26" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="B26" s="8">
+      <c r="B26" s="6">
         <f>B24+B21</f>
         <v>707192</v>
       </c>
-      <c r="C26" s="18">
+      <c r="C26" s="13">
         <f>C21+C25</f>
         <v>727739.72602739721</v>
       </c>
-      <c r="D26" s="18">
+      <c r="D26" s="13">
         <f t="shared" ref="D26:E26" si="9">D21+D25</f>
         <v>753424.65753424657</v>
       </c>
-      <c r="E26" s="18">
+      <c r="E26" s="13">
         <f t="shared" si="9"/>
         <v>785530.82191780815</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A27" s="5"/>
-      <c r="B27" s="7"/>
+      <c r="A27" s="3"/>
+      <c r="B27" s="5"/>
     </row>
     <row r="28" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A28" s="6" t="s">
+      <c r="A28" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="B28" s="7"/>
+      <c r="B28" s="5"/>
     </row>
     <row r="29" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A29" s="5" t="s">
+      <c r="A29" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="B29" s="7">
+      <c r="B29" s="5">
         <v>1000000</v>
       </c>
-      <c r="C29" s="16">
+      <c r="C29" s="11">
         <f>B29</f>
         <v>1000000</v>
       </c>
-      <c r="D29" s="16">
+      <c r="D29" s="11">
         <f t="shared" ref="D29:E29" si="10">C29</f>
         <v>1000000</v>
       </c>
-      <c r="E29" s="16">
+      <c r="E29" s="11">
         <f t="shared" si="10"/>
         <v>1000000</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A30" s="5" t="s">
+      <c r="A30" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="B30" s="7">
+      <c r="B30" s="5">
         <v>1309246</v>
       </c>
-      <c r="C30" s="16">
+      <c r="C30" s="11">
         <f>B30+'Income statement '!C22</f>
         <v>2106121</v>
       </c>
-      <c r="D30" s="16">
+      <c r="D30" s="11">
         <f>C30+'Income statement '!D22</f>
         <v>3242839.75</v>
       </c>
-      <c r="E30" s="16">
+      <c r="E30" s="11">
         <f>D30+'Income statement '!E22</f>
         <v>4804363.1875</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A31" s="6" t="s">
+      <c r="A31" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B31" s="8">
+      <c r="B31" s="6">
         <f>SUM(B29:B30)</f>
         <v>2309246</v>
       </c>
-      <c r="C31" s="16">
+      <c r="C31" s="11">
         <f>SUM(C29:C30)</f>
         <v>3106121</v>
       </c>
-      <c r="D31" s="16">
+      <c r="D31" s="11">
         <f t="shared" ref="D31:E31" si="11">SUM(D29:D30)</f>
         <v>4242839.75</v>
       </c>
-      <c r="E31" s="16">
+      <c r="E31" s="11">
         <f t="shared" si="11"/>
         <v>5804363.1875</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A32" s="14" t="s">
+      <c r="A32" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="B32" s="15">
+      <c r="B32" s="10">
         <f>B26+B31</f>
         <v>3016438</v>
       </c>
-      <c r="C32" s="17">
+      <c r="C32" s="12">
         <f>C26+C31</f>
         <v>3833860.7260273974</v>
       </c>
-      <c r="D32" s="17">
+      <c r="D32" s="12">
         <f t="shared" ref="D32:E32" si="12">D26+D31</f>
         <v>4996264.4075342463</v>
       </c>
-      <c r="E32" s="17">
+      <c r="E32" s="12">
         <f t="shared" si="12"/>
         <v>6589894.0094178077</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="A1:E2"/>
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="C3:C4"/>
     <mergeCell ref="D3:D4"/>
     <mergeCell ref="E3:E4"/>
     <mergeCell ref="A3:A4"/>
-    <mergeCell ref="A1:E2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1992,18 +2143,500 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88E1F010-C4FB-4CC3-82AF-6E4EB4905CC1}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="67.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="5" width="10.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="32" t="s">
+        <v>68</v>
+      </c>
+      <c r="B3" s="32" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="32" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" s="32" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" s="32" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="31" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>70</v>
+      </c>
+      <c r="B5" s="40">
+        <f>'Income statement '!B11</f>
+        <v>1250000</v>
+      </c>
+      <c r="C5" s="40">
+        <f>'Income statement '!C11</f>
+        <v>1562500</v>
+      </c>
+      <c r="D5" s="40">
+        <f>'Income statement '!D11</f>
+        <v>1953125</v>
+      </c>
+      <c r="E5" s="40">
+        <f>'Income statement '!E11</f>
+        <v>2441406.25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B6" s="40">
+        <f>'Income statement '!B7</f>
+        <v>5000000</v>
+      </c>
+      <c r="C6" s="40">
+        <f>'Income statement '!C7</f>
+        <v>6250000</v>
+      </c>
+      <c r="D6" s="40">
+        <f>'Income statement '!D7</f>
+        <v>7812500</v>
+      </c>
+      <c r="E6" s="40">
+        <f>'Income statement '!E7</f>
+        <v>9765625</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>72</v>
+      </c>
+      <c r="B7" s="40">
+        <v>0</v>
+      </c>
+      <c r="C7" s="40">
+        <v>123288</v>
+      </c>
+      <c r="D7" s="40">
+        <v>-102739</v>
+      </c>
+      <c r="E7" s="40">
+        <v>-128425</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="33" t="s">
+        <v>73</v>
+      </c>
+      <c r="B8" s="41">
+        <f>SUM(B5:B7)</f>
+        <v>6250000</v>
+      </c>
+      <c r="C8" s="41">
+        <f>SUM(C5:C7)</f>
+        <v>7935788</v>
+      </c>
+      <c r="D8" s="41">
+        <f>SUM(D5:D7)</f>
+        <v>9662886</v>
+      </c>
+      <c r="E8" s="41">
+        <f>SUM(E5:E7)</f>
+        <v>12078606.25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B9" s="40"/>
+      <c r="C9" s="40"/>
+      <c r="D9" s="40"/>
+      <c r="E9" s="40"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" s="31" t="s">
+        <v>74</v>
+      </c>
+      <c r="B10" s="40"/>
+      <c r="C10" s="40"/>
+      <c r="D10" s="40"/>
+      <c r="E10" s="40"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>75</v>
+      </c>
+      <c r="B11" s="40">
+        <v>0</v>
+      </c>
+      <c r="C11" s="40">
+        <v>0</v>
+      </c>
+      <c r="D11" s="40">
+        <v>0</v>
+      </c>
+      <c r="E11" s="40">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="31" t="s">
+        <v>76</v>
+      </c>
+      <c r="B12" s="56">
+        <v>0</v>
+      </c>
+      <c r="C12" s="56">
+        <v>0</v>
+      </c>
+      <c r="D12" s="56">
+        <v>0</v>
+      </c>
+      <c r="E12" s="56">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B13" s="40"/>
+      <c r="C13" s="40"/>
+      <c r="D13" s="40"/>
+      <c r="E13" s="40"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" s="31" t="s">
+        <v>77</v>
+      </c>
+      <c r="B14" s="40"/>
+      <c r="C14" s="40"/>
+      <c r="D14" s="40"/>
+      <c r="E14" s="40"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>78</v>
+      </c>
+      <c r="B15" s="40">
+        <v>0</v>
+      </c>
+      <c r="C15" s="40">
+        <v>0</v>
+      </c>
+      <c r="D15" s="40">
+        <v>0</v>
+      </c>
+      <c r="E15" s="40">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" s="31" t="s">
+        <v>79</v>
+      </c>
+      <c r="B16" s="56">
+        <v>0</v>
+      </c>
+      <c r="C16" s="56">
+        <v>0</v>
+      </c>
+      <c r="D16" s="56">
+        <v>0</v>
+      </c>
+      <c r="E16" s="56">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B17" s="40"/>
+      <c r="C17" s="40"/>
+      <c r="D17" s="40"/>
+      <c r="E17" s="40"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="B18" s="42">
+        <f>B8+B12+B16</f>
+        <v>6250000</v>
+      </c>
+      <c r="C18" s="42">
+        <f>C8+C12+C16</f>
+        <v>7935788</v>
+      </c>
+      <c r="D18" s="42">
+        <f>D8+D12+D16</f>
+        <v>9662886</v>
+      </c>
+      <c r="E18" s="42">
+        <f>E8+E12+E16</f>
+        <v>12078606.25</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>81</v>
+      </c>
+      <c r="B19" s="40">
+        <v>0</v>
+      </c>
+      <c r="C19" s="40">
+        <f>B20</f>
+        <v>6250000</v>
+      </c>
+      <c r="D19" s="40">
+        <f>C20</f>
+        <v>14185788</v>
+      </c>
+      <c r="E19" s="40">
+        <f>D20</f>
+        <v>23848674</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" s="35" t="s">
+        <v>82</v>
+      </c>
+      <c r="B20" s="43">
+        <f>B18+B19</f>
+        <v>6250000</v>
+      </c>
+      <c r="C20" s="43">
+        <f>C18+C19</f>
+        <v>14185788</v>
+      </c>
+      <c r="D20" s="43">
+        <f>D18+D19</f>
+        <v>23848674</v>
+      </c>
+      <c r="E20" s="43">
+        <f>E18+E19</f>
+        <v>35927280.25</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27EA545A-387F-4AE1-B78E-057214D5B253}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="62.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="6" width="11.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="32" t="s">
+        <v>84</v>
+      </c>
+      <c r="B3" s="32" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B4" s="40">
+        <f>'Income statement '!E6</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>87</v>
+      </c>
+      <c r="B5" s="36">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>88</v>
+      </c>
+      <c r="B6" s="36">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>89</v>
+      </c>
+      <c r="B7" s="36">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" s="37" t="s">
+        <v>90</v>
+      </c>
+      <c r="B8" s="44">
+        <v>19238543</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="31" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" s="38" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="32" t="s">
+        <v>93</v>
+      </c>
+      <c r="B14" s="39">
+        <v>0.02</v>
+      </c>
+      <c r="C14" s="39">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="D14" s="39">
+        <v>0.03</v>
+      </c>
+      <c r="E14" s="39">
+        <v>3.5000000000000003E-2</v>
+      </c>
+      <c r="F14" s="39">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" s="39"/>
+      <c r="B15" s="45">
+        <f>ROUND(19238543 * (((1+B$14)/($A15-B$14))/((1+0.03)/(0.1-0.03))), 0)</f>
+        <v>-66681164</v>
+      </c>
+      <c r="C15" s="45">
+        <f>ROUND(19238543 * (((1+C$14)/($A15-C$14))/((1+0.03)/(0.1-0.03))), 0)</f>
+        <v>-53606426</v>
+      </c>
+      <c r="D15" s="45">
+        <f>ROUND(19238543 * (((1+D$14)/($A15-D$14))/((1+0.03)/(0.1-0.03))), 0)</f>
+        <v>-44889934</v>
+      </c>
+      <c r="E15" s="45">
+        <f>ROUND(19238543 * (((1+E$14)/($A15-E$14))/((1+0.03)/(0.1-0.03))), 0)</f>
+        <v>-38663868</v>
+      </c>
+      <c r="F15" s="45">
+        <f>ROUND(19238543 * (((1+F$14)/($A15-F$14))/((1+0.03)/(0.1-0.03))), 0)</f>
+        <v>-33994319</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="39"/>
+      <c r="B16" s="45">
+        <f>ROUND(19238543 * (((1+B$14)/($A16-B$14))/((1+0.03)/(0.1-0.03))), 0)</f>
+        <v>-66681164</v>
+      </c>
+      <c r="C16" s="45">
+        <f>ROUND(19238543 * (((1+C$14)/($A16-C$14))/((1+0.03)/(0.1-0.03))), 0)</f>
+        <v>-53606426</v>
+      </c>
+      <c r="D16" s="45">
+        <f>ROUND(19238543 * (((1+D$14)/($A16-D$14))/((1+0.03)/(0.1-0.03))), 0)</f>
+        <v>-44889934</v>
+      </c>
+      <c r="E16" s="45">
+        <f>ROUND(19238543 * (((1+E$14)/($A16-E$14))/((1+0.03)/(0.1-0.03))), 0)</f>
+        <v>-38663868</v>
+      </c>
+      <c r="F16" s="45">
+        <f>ROUND(19238543 * (((1+F$14)/($A16-F$14))/((1+0.03)/(0.1-0.03))), 0)</f>
+        <v>-33994319</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="39"/>
+      <c r="B17" s="46">
+        <f>ROUND(19238543 * (((1+B$14)/($A17-B$14))/((1+0.03)/(0.1-0.03))), 0)</f>
+        <v>-66681164</v>
+      </c>
+      <c r="C17" s="46">
+        <f>ROUND(19238543 * (((1+C$14)/($A17-C$14))/((1+0.03)/(0.1-0.03))), 0)</f>
+        <v>-53606426</v>
+      </c>
+      <c r="D17" s="44">
+        <f>ROUND(19238543 * (((1+D$14)/($A17-D$14))/((1+0.03)/(0.1-0.03))), 0)</f>
+        <v>-44889934</v>
+      </c>
+      <c r="E17" s="45">
+        <f>ROUND(19238543 * (((1+E$14)/($A17-E$14))/((1+0.03)/(0.1-0.03))), 0)</f>
+        <v>-38663868</v>
+      </c>
+      <c r="F17" s="45">
+        <f>ROUND(19238543 * (((1+F$14)/($A17-F$14))/((1+0.03)/(0.1-0.03))), 0)</f>
+        <v>-33994319</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" s="39"/>
+      <c r="B18" s="46">
+        <f>ROUND(19238543 * (((1+B$14)/($A18-B$14))/((1+0.03)/(0.1-0.03))), 0)</f>
+        <v>-66681164</v>
+      </c>
+      <c r="C18" s="46">
+        <f>ROUND(19238543 * (((1+C$14)/($A18-C$14))/((1+0.03)/(0.1-0.03))), 0)</f>
+        <v>-53606426</v>
+      </c>
+      <c r="D18" s="46">
+        <f>ROUND(19238543 * (((1+D$14)/($A18-D$14))/((1+0.03)/(0.1-0.03))), 0)</f>
+        <v>-44889934</v>
+      </c>
+      <c r="E18" s="45">
+        <f>ROUND(19238543 * (((1+E$14)/($A18-E$14))/((1+0.03)/(0.1-0.03))), 0)</f>
+        <v>-38663868</v>
+      </c>
+      <c r="F18" s="45">
+        <f>ROUND(19238543 * (((1+F$14)/($A18-F$14))/((1+0.03)/(0.1-0.03))), 0)</f>
+        <v>-33994319</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" s="39"/>
+      <c r="B19" s="46">
+        <f>ROUND(19238543 * (((1+B$14)/($A19-B$14))/((1+0.03)/(0.1-0.03))), 0)</f>
+        <v>-66681164</v>
+      </c>
+      <c r="C19" s="46">
+        <f>ROUND(19238543 * (((1+C$14)/($A19-C$14))/((1+0.03)/(0.1-0.03))), 0)</f>
+        <v>-53606426</v>
+      </c>
+      <c r="D19" s="46">
+        <f>ROUND(19238543 * (((1+D$14)/($A19-D$14))/((1+0.03)/(0.1-0.03))), 0)</f>
+        <v>-44889934</v>
+      </c>
+      <c r="E19" s="45">
+        <f>ROUND(19238543 * (((1+E$14)/($A19-E$14))/((1+0.03)/(0.1-0.03))), 0)</f>
+        <v>-38663868</v>
+      </c>
+      <c r="F19" s="45">
+        <f>ROUND(19238543 * (((1+F$14)/($A19-F$14))/((1+0.03)/(0.1-0.03))), 0)</f>
+        <v>-33994319</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>